<commit_message>
feat: UrbanPiper aggregator, customer auto-merge, table system settings, support step-up access, super-admin employees and email approvals
Also includes KDS rollup, order/menu notifiers, mail fallback, SEO tweaks, QA docs refresh, and Prisma migrations for support login credentials, complimentary subscriptions, staff soft delete and approval email tokens.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/qa/export/excel/TEST_RUN_SHEET.xlsx
+++ b/docs/qa/export/excel/TEST_RUN_SHEET.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="704">
   <si>
     <t>Field</t>
   </si>
@@ -785,6 +785,96 @@
     <t>Kiosk order placed</t>
   </si>
   <si>
+    <t>TC-2.8-01</t>
+  </si>
+  <si>
+    <t>2.8 Web kiosk</t>
+  </si>
+  <si>
+    <t>Kiosk opens at kiosk.cullinos.com/o/{org}/{outlet} on welcome screen</t>
+  </si>
+  <si>
+    <t>Welcome screen</t>
+  </si>
+  <si>
+    <t>TC-2.8-02</t>
+  </si>
+  <si>
+    <t>Start → add item with modifiers to cart</t>
+  </si>
+  <si>
+    <t>Item + modifiers in cart</t>
+  </si>
+  <si>
+    <t>TC-2.8-03</t>
+  </si>
+  <si>
+    <t>Place order shows pickup code</t>
+  </si>
+  <si>
+    <t>Pickup code shown</t>
+  </si>
+  <si>
+    <t>TC-2.8-04</t>
+  </si>
+  <si>
+    <t>Kiosk order appears in POS / KDS</t>
+  </si>
+  <si>
+    <t>Order in POS/KDS</t>
+  </si>
+  <si>
+    <t>TC-2.8-05</t>
+  </si>
+  <si>
+    <t>Idle ~2 min returns to welcome screen</t>
+  </si>
+  <si>
+    <t>TC-2.9-01</t>
+  </si>
+  <si>
+    <t>2.9 Token ordering</t>
+  </si>
+  <si>
+    <t>Counter QR card shown (Settings / /kiosk) when table system is off</t>
+  </si>
+  <si>
+    <t>Counter QR visible</t>
+  </si>
+  <si>
+    <t>TC-2.9-02</t>
+  </si>
+  <si>
+    <t>Guest picks Eat in / Takeaway and places order</t>
+  </si>
+  <si>
+    <t>TC-2.9-03</t>
+  </si>
+  <si>
+    <t>Guest sees Your token (pickup code) + order number</t>
+  </si>
+  <si>
+    <t>Token shown</t>
+  </si>
+  <si>
+    <t>TC-2.9-04</t>
+  </si>
+  <si>
+    <t>KDS ticket shows Token XXXXXX (no table)</t>
+  </si>
+  <si>
+    <t>Token on KDS</t>
+  </si>
+  <si>
+    <t>TC-2.9-05</t>
+  </si>
+  <si>
+    <t>Pickup / CDS display lists the same token</t>
+  </si>
+  <si>
+    <t>Token on CDS</t>
+  </si>
+  <si>
     <t>TC-3-01</t>
   </si>
   <si>
@@ -1181,6 +1271,114 @@
     <t>Export works</t>
   </si>
   <si>
+    <t>TC-3-46</t>
+  </si>
+  <si>
+    <t>Settings → Table system off — Tables / Reservations leave nav for outlet</t>
+  </si>
+  <si>
+    <t>Nav hidden</t>
+  </si>
+  <si>
+    <t>TC-3-47</t>
+  </si>
+  <si>
+    <t>Table system off — table QR shows counter flow; new table session rejected</t>
+  </si>
+  <si>
+    <t>Counter flow; session rejected</t>
+  </si>
+  <si>
+    <t>TC-3-48</t>
+  </si>
+  <si>
+    <t>Table system on / "Use category default" — Tables nav and table sessions work</t>
+  </si>
+  <si>
+    <t>Tables work</t>
+  </si>
+  <si>
+    <t>TC-3-49</t>
+  </si>
+  <si>
+    <t>Aggregators — UrbanPiper connect saves; webhook URL + secret shown</t>
+  </si>
+  <si>
+    <t>Connected</t>
+  </si>
+  <si>
+    <t>TC-3-50</t>
+  </si>
+  <si>
+    <t>Aggregators — per-outlet store link + menu push (or graceful error)</t>
+  </si>
+  <si>
+    <t>Push OK or clear error</t>
+  </si>
+  <si>
+    <t>TC-3-51</t>
+  </si>
+  <si>
+    <t>Aggregators — store pause / per-outlet item stock toggle</t>
+  </si>
+  <si>
+    <t>Toggles persist</t>
+  </si>
+  <si>
+    <t>TC-3-52</t>
+  </si>
+  <si>
+    <t>Aggregators — unknown-item linking + settlement CSV import</t>
+  </si>
+  <si>
+    <t>Linked; CSV imported</t>
+  </si>
+  <si>
+    <t>TC-3-53</t>
+  </si>
+  <si>
+    <t>Portal POS Online panel loads; new order chimes with accept timer (or N/A)</t>
+  </si>
+  <si>
+    <t>Panel OK or N/A</t>
+  </si>
+  <si>
+    <t>TC-3-54</t>
+  </si>
+  <si>
+    <t>Online panel — Accept (prep time) prints KOT; Reject requires reason</t>
+  </si>
+  <si>
+    <t>KOT on accept; reason enforced</t>
+  </si>
+  <si>
+    <t>TC-3-55</t>
+  </si>
+  <si>
+    <t>Online panel — Food ready → Handed to rider</t>
+  </si>
+  <si>
+    <t>Status advances</t>
+  </si>
+  <si>
+    <t>TC-3-56</t>
+  </si>
+  <si>
+    <t>Customers — Find duplicates shows merge preview</t>
+  </si>
+  <si>
+    <t>Preview shown</t>
+  </si>
+  <si>
+    <t>TC-3-57</t>
+  </si>
+  <si>
+    <t>Customers — Apply merge combines duplicates</t>
+  </si>
+  <si>
+    <t>Duplicates merged</t>
+  </si>
+  <si>
     <t>TC-4-01</t>
   </si>
   <si>
@@ -1409,7 +1607,7 @@
     <t>TC-5-21</t>
   </si>
   <si>
-    <t>Guest Ops overview loads</t>
+    <t>Guest Ops (App Ops) overview loads</t>
   </si>
   <si>
     <t>Overview loads</t>
@@ -1418,7 +1616,7 @@
     <t>TC-5-22</t>
   </si>
   <si>
-    <t>Guest Ops marketplace — approve/rank QA listing</t>
+    <t>Guest Ops (App Ops) marketplace — approve/rank QA listing</t>
   </si>
   <si>
     <t>Listing updated</t>
@@ -1427,7 +1625,7 @@
     <t>TC-5-23</t>
   </si>
   <si>
-    <t>Guest Ops discover — create section</t>
+    <t>Guest Ops (App Ops) discover — create section</t>
   </si>
   <si>
     <t>Section created</t>
@@ -1436,28 +1634,28 @@
     <t>TC-5-24</t>
   </si>
   <si>
-    <t>Guest Ops banners — create banner</t>
+    <t>Guest Ops (App Ops) banners — create banner</t>
   </si>
   <si>
     <t>TC-5-25</t>
   </si>
   <si>
-    <t>Guest Ops push — create draft</t>
+    <t>Guest Ops (App Ops) notifications — create draft</t>
   </si>
   <si>
     <t>TC-5-26</t>
   </si>
   <si>
-    <t>Guest Ops offers — create offer</t>
-  </si>
-  <si>
-    <t>Offer created</t>
+    <t>Guest Ops offers — create offer (N/A if route redirects home)</t>
+  </si>
+  <si>
+    <t>Offer created or N/A</t>
   </si>
   <si>
     <t>TC-5-27</t>
   </si>
   <si>
-    <t>Guest Ops reviews / users / analytics pages load</t>
+    <t>Guest Ops (App Ops) reviews / users / analytics pages load</t>
   </si>
   <si>
     <t>Pages load</t>
@@ -1466,7 +1664,7 @@
     <t>TC-5-28</t>
   </si>
   <si>
-    <t>Guest Ops runtime — Save runtime settings (safe toggle)</t>
+    <t>Guest Ops (App Ops) runtime — Save runtime settings (safe toggle)</t>
   </si>
   <si>
     <t>TC-5-29</t>
@@ -1487,6 +1685,57 @@
     <t>Impersonation works</t>
   </si>
   <si>
+    <t>TC-5-31</t>
+  </si>
+  <si>
+    <t>Employees page lists platform employees</t>
+  </si>
+  <si>
+    <t>List loads</t>
+  </si>
+  <si>
+    <t>TC-5-32</t>
+  </si>
+  <si>
+    <t>Employees — Onboard employee dialog submits (QA email, human approval)</t>
+  </si>
+  <si>
+    <t>Employee invited</t>
+  </si>
+  <si>
+    <t>TC-5-33</t>
+  </si>
+  <si>
+    <t>Approvals inbox loads; approval detail opens</t>
+  </si>
+  <si>
+    <t>Inbox + detail load</t>
+  </si>
+  <si>
+    <t>TC-5-34</t>
+  </si>
+  <si>
+    <t>Approvals policies page loads</t>
+  </si>
+  <si>
+    <t>TC-5-35</t>
+  </si>
+  <si>
+    <t>Approval email-action link opens approval page</t>
+  </si>
+  <si>
+    <t>TC-5-36</t>
+  </si>
+  <si>
+    <t>People directory and org chart load</t>
+  </si>
+  <si>
+    <t>TC-5-37</t>
+  </si>
+  <si>
+    <t>Employee profile page opens</t>
+  </si>
+  <si>
     <t>TC-6-01</t>
   </si>
   <si>
@@ -1706,6 +1955,108 @@
     <t>Integrations — list</t>
   </si>
   <si>
+    <t>TC-8-01</t>
+  </si>
+  <si>
+    <t>8 Support</t>
+  </si>
+  <si>
+    <t>Restaurant login with owner credentials (OTP if prompted)</t>
+  </si>
+  <si>
+    <t>Portal home loads</t>
+  </si>
+  <si>
+    <t>TC-8-02</t>
+  </si>
+  <si>
+    <t>Portal home loads; KB article opens</t>
+  </si>
+  <si>
+    <t>TC-8-03</t>
+  </si>
+  <si>
+    <t>Raise ticket submits; appears in My tickets</t>
+  </si>
+  <si>
+    <t>Ticket listed</t>
+  </si>
+  <si>
+    <t>TC-8-04</t>
+  </si>
+  <si>
+    <t>Ticket detail — reply posts</t>
+  </si>
+  <si>
+    <t>Reply visible</t>
+  </si>
+  <si>
+    <t>TC-8-05</t>
+  </si>
+  <si>
+    <t>Agent login (Rkyves staff) lands on queue</t>
+  </si>
+  <si>
+    <t>Queue loads</t>
+  </si>
+  <si>
+    <t>TC-8-06</t>
+  </si>
+  <si>
+    <t>Agent opens QA tenant ticket and replies</t>
+  </si>
+  <si>
+    <t>Reply visible to tenant</t>
+  </si>
+  <si>
+    <t>TC-8-07</t>
+  </si>
+  <si>
+    <t>Agent dashboard loads</t>
+  </si>
+  <si>
+    <t>TC-8-08</t>
+  </si>
+  <si>
+    <t>Agent grants — tenant access request prompts step-up</t>
+  </si>
+  <si>
+    <t>Step-up dialog shown</t>
+  </si>
+  <si>
+    <t>TC-8-09</t>
+  </si>
+  <si>
+    <t>Agent shifts page loads</t>
+  </si>
+  <si>
+    <t>TC-8-10</t>
+  </si>
+  <si>
+    <t>Agent knowledge page loads</t>
+  </si>
+  <si>
+    <t>TC-9-01</t>
+  </si>
+  <si>
+    <t>9 App Ops</t>
+  </si>
+  <si>
+    <t>App Ops login succeeds</t>
+  </si>
+  <si>
+    <t>TC-9-02</t>
+  </si>
+  <si>
+    <t>Super Admin /guest-ops redirects to App Ops</t>
+  </si>
+  <si>
+    <t>TC-9-03</t>
+  </si>
+  <si>
+    <t>App Ops forgot-password page loads</t>
+  </si>
+  <si>
     <t>Count</t>
   </si>
   <si>
@@ -1742,7 +2093,7 @@
     <t>Known limitations separated from open bugs</t>
   </si>
   <si>
-    <t>All 190 test cases marked Pass/Fail/Blocked/N/A</t>
+    <t>All 232 test cases marked Pass/Fail/Blocked/N/A</t>
   </si>
   <si>
     <t>Tester signature</t>
@@ -1775,7 +2126,7 @@
     <t>5. Complete Sign-off sheet on last day.</t>
   </si>
   <si>
-    <t>Total test cases: 190</t>
+    <t>Total test cases: 232</t>
   </si>
 </sst>
 </file>
@@ -2261,7 +2612,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G191"/>
+  <dimension ref="A1:G233"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -3441,15 +3792,15 @@
         <v>270</v>
       </c>
       <c r="D83" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>271</v>
+      </c>
+      <c r="B84" t="s">
         <v>272</v>
-      </c>
-      <c r="B84" t="s">
-        <v>257</v>
       </c>
       <c r="C84" t="s">
         <v>273</v>
@@ -3463,63 +3814,63 @@
         <v>275</v>
       </c>
       <c r="B85" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="C85" t="s">
         <v>276</v>
       </c>
       <c r="D85" t="s">
-        <v>277</v>
+        <v>179</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>277</v>
+      </c>
+      <c r="B86" t="s">
+        <v>272</v>
+      </c>
+      <c r="C86" t="s">
         <v>278</v>
       </c>
-      <c r="B86" t="s">
-        <v>257</v>
-      </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
         <v>279</v>
-      </c>
-      <c r="D86" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>280</v>
+      </c>
+      <c r="B87" t="s">
+        <v>272</v>
+      </c>
+      <c r="C87" t="s">
         <v>281</v>
       </c>
-      <c r="B87" t="s">
-        <v>257</v>
-      </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
         <v>282</v>
-      </c>
-      <c r="D87" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>283</v>
+      </c>
+      <c r="B88" t="s">
+        <v>272</v>
+      </c>
+      <c r="C88" t="s">
         <v>284</v>
       </c>
-      <c r="B88" t="s">
-        <v>257</v>
-      </c>
-      <c r="C88" t="s">
+      <c r="D88" t="s">
         <v>285</v>
-      </c>
-      <c r="D88" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>286</v>
+      </c>
+      <c r="B89" t="s">
         <v>287</v>
-      </c>
-      <c r="B89" t="s">
-        <v>257</v>
       </c>
       <c r="C89" t="s">
         <v>288</v>
@@ -3533,7 +3884,7 @@
         <v>290</v>
       </c>
       <c r="B90" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C90" t="s">
         <v>291</v>
@@ -3547,7 +3898,7 @@
         <v>293</v>
       </c>
       <c r="B91" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C91" t="s">
         <v>294</v>
@@ -3561,7 +3912,7 @@
         <v>296</v>
       </c>
       <c r="B92" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C92" t="s">
         <v>297</v>
@@ -3575,7 +3926,7 @@
         <v>299</v>
       </c>
       <c r="B93" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C93" t="s">
         <v>300</v>
@@ -3589,7 +3940,7 @@
         <v>302</v>
       </c>
       <c r="B94" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C94" t="s">
         <v>303</v>
@@ -3603,7 +3954,7 @@
         <v>305</v>
       </c>
       <c r="B95" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C95" t="s">
         <v>306</v>
@@ -3617,7 +3968,7 @@
         <v>308</v>
       </c>
       <c r="B96" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C96" t="s">
         <v>309</v>
@@ -3631,7 +3982,7 @@
         <v>311</v>
       </c>
       <c r="B97" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C97" t="s">
         <v>312</v>
@@ -3645,7 +3996,7 @@
         <v>314</v>
       </c>
       <c r="B98" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C98" t="s">
         <v>315</v>
@@ -3659,7 +4010,7 @@
         <v>317</v>
       </c>
       <c r="B99" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C99" t="s">
         <v>318</v>
@@ -3673,7 +4024,7 @@
         <v>320</v>
       </c>
       <c r="B100" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C100" t="s">
         <v>321</v>
@@ -3687,7 +4038,7 @@
         <v>323</v>
       </c>
       <c r="B101" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C101" t="s">
         <v>324</v>
@@ -3701,7 +4052,7 @@
         <v>326</v>
       </c>
       <c r="B102" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C102" t="s">
         <v>327</v>
@@ -3715,7 +4066,7 @@
         <v>329</v>
       </c>
       <c r="B103" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C103" t="s">
         <v>330</v>
@@ -3729,7 +4080,7 @@
         <v>332</v>
       </c>
       <c r="B104" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C104" t="s">
         <v>333</v>
@@ -3743,7 +4094,7 @@
         <v>335</v>
       </c>
       <c r="B105" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C105" t="s">
         <v>336</v>
@@ -3757,7 +4108,7 @@
         <v>338</v>
       </c>
       <c r="B106" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C106" t="s">
         <v>339</v>
@@ -3771,220 +4122,220 @@
         <v>341</v>
       </c>
       <c r="B107" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C107" t="s">
         <v>342</v>
       </c>
       <c r="D107" t="s">
-        <v>105</v>
+        <v>343</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B108" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C108" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D108" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B109" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C109" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D109" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B110" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C110" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D110" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B111" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C111" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D111" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B112" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C112" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D112" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B113" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C113" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D113" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B114" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C114" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="D114" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B115" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C115" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="D115" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B116" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C116" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="D116" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="B117" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C117" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="D117" t="s">
-        <v>369</v>
+        <v>105</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B118" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C118" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="D118" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B119" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C119" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D119" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B120" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C120" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="D120" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B121" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C121" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="D121" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B122" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C122" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="D122" t="s">
         <v>384</v>
@@ -3992,114 +4343,114 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B123" t="s">
-        <v>257</v>
+        <v>287</v>
       </c>
       <c r="C123" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D123" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B124" t="s">
-        <v>389</v>
+        <v>287</v>
       </c>
       <c r="C124" t="s">
         <v>390</v>
       </c>
       <c r="D124" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
+        <v>391</v>
+      </c>
+      <c r="B125" t="s">
+        <v>287</v>
+      </c>
+      <c r="C125" t="s">
         <v>392</v>
       </c>
-      <c r="B125" t="s">
-        <v>389</v>
-      </c>
-      <c r="C125" t="s">
+      <c r="D125" t="s">
         <v>393</v>
-      </c>
-      <c r="D125" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
+        <v>394</v>
+      </c>
+      <c r="B126" t="s">
+        <v>287</v>
+      </c>
+      <c r="C126" t="s">
         <v>395</v>
       </c>
-      <c r="B126" t="s">
-        <v>389</v>
-      </c>
-      <c r="C126" t="s">
+      <c r="D126" t="s">
         <v>396</v>
-      </c>
-      <c r="D126" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
+        <v>397</v>
+      </c>
+      <c r="B127" t="s">
+        <v>287</v>
+      </c>
+      <c r="C127" t="s">
         <v>398</v>
       </c>
-      <c r="B127" t="s">
-        <v>389</v>
-      </c>
-      <c r="C127" t="s">
+      <c r="D127" t="s">
         <v>399</v>
-      </c>
-      <c r="D127" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
+        <v>400</v>
+      </c>
+      <c r="B128" t="s">
+        <v>287</v>
+      </c>
+      <c r="C128" t="s">
         <v>401</v>
       </c>
-      <c r="B128" t="s">
-        <v>389</v>
-      </c>
-      <c r="C128" t="s">
+      <c r="D128" t="s">
         <v>402</v>
-      </c>
-      <c r="D128" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
+        <v>403</v>
+      </c>
+      <c r="B129" t="s">
+        <v>287</v>
+      </c>
+      <c r="C129" t="s">
         <v>404</v>
       </c>
-      <c r="B129" t="s">
-        <v>389</v>
-      </c>
-      <c r="C129" t="s">
+      <c r="D129" t="s">
         <v>405</v>
-      </c>
-      <c r="D129" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
+        <v>406</v>
+      </c>
+      <c r="B130" t="s">
+        <v>287</v>
+      </c>
+      <c r="C130" t="s">
         <v>407</v>
       </c>
-      <c r="B130" t="s">
-        <v>389</v>
-      </c>
-      <c r="C130" t="s">
+      <c r="D130" t="s">
         <v>408</v>
-      </c>
-      <c r="D130" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
@@ -4107,7 +4458,7 @@
         <v>409</v>
       </c>
       <c r="B131" t="s">
-        <v>389</v>
+        <v>287</v>
       </c>
       <c r="C131" t="s">
         <v>410</v>
@@ -4121,69 +4472,69 @@
         <v>412</v>
       </c>
       <c r="B132" t="s">
+        <v>287</v>
+      </c>
+      <c r="C132" t="s">
         <v>413</v>
       </c>
-      <c r="C132" t="s">
+      <c r="D132" t="s">
         <v>414</v>
-      </c>
-      <c r="D132" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
+        <v>415</v>
+      </c>
+      <c r="B133" t="s">
+        <v>287</v>
+      </c>
+      <c r="C133" t="s">
         <v>416</v>
       </c>
-      <c r="B133" t="s">
-        <v>413</v>
-      </c>
-      <c r="C133" t="s">
+      <c r="D133" t="s">
         <v>417</v>
-      </c>
-      <c r="D133" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
+        <v>418</v>
+      </c>
+      <c r="B134" t="s">
+        <v>287</v>
+      </c>
+      <c r="C134" t="s">
         <v>419</v>
       </c>
-      <c r="B134" t="s">
-        <v>413</v>
-      </c>
-      <c r="C134" t="s">
+      <c r="D134" t="s">
         <v>420</v>
-      </c>
-      <c r="D134" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
+        <v>421</v>
+      </c>
+      <c r="B135" t="s">
+        <v>287</v>
+      </c>
+      <c r="C135" t="s">
         <v>422</v>
       </c>
-      <c r="B135" t="s">
-        <v>413</v>
-      </c>
-      <c r="C135" t="s">
+      <c r="D135" t="s">
         <v>423</v>
-      </c>
-      <c r="D135" t="s">
-        <v>424</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
+        <v>424</v>
+      </c>
+      <c r="B136" t="s">
+        <v>287</v>
+      </c>
+      <c r="C136" t="s">
         <v>425</v>
       </c>
-      <c r="B136" t="s">
-        <v>413</v>
-      </c>
-      <c r="C136" t="s">
+      <c r="D136" t="s">
         <v>426</v>
-      </c>
-      <c r="D136" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
@@ -4191,7 +4542,7 @@
         <v>427</v>
       </c>
       <c r="B137" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C137" t="s">
         <v>428</v>
@@ -4205,7 +4556,7 @@
         <v>430</v>
       </c>
       <c r="B138" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C138" t="s">
         <v>431</v>
@@ -4219,472 +4570,472 @@
         <v>433</v>
       </c>
       <c r="B139" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C139" t="s">
         <v>434</v>
       </c>
       <c r="D139" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B140" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C140" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D140" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B141" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C141" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D141" t="s">
-        <v>432</v>
+        <v>441</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B142" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C142" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="D142" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B143" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C143" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="D143" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="B144" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C144" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="D144" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B145" t="s">
-        <v>413</v>
+        <v>287</v>
       </c>
       <c r="C145" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="D145" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B146" t="s">
-        <v>413</v>
+        <v>455</v>
       </c>
       <c r="C146" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="D146" t="s">
-        <v>105</v>
+        <v>457</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="B147" t="s">
-        <v>413</v>
+        <v>455</v>
       </c>
       <c r="C147" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="D147" t="s">
-        <v>105</v>
+        <v>460</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
+        <v>461</v>
+      </c>
+      <c r="B148" t="s">
         <v>455</v>
       </c>
-      <c r="B148" t="s">
-        <v>413</v>
-      </c>
       <c r="C148" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="D148" t="s">
-        <v>432</v>
+        <v>463</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="B149" t="s">
-        <v>413</v>
+        <v>455</v>
       </c>
       <c r="C149" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="D149" t="s">
-        <v>105</v>
+        <v>466</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="B150" t="s">
-        <v>413</v>
+        <v>455</v>
       </c>
       <c r="C150" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
       <c r="D150" t="s">
-        <v>105</v>
+        <v>469</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B151" t="s">
-        <v>413</v>
+        <v>455</v>
       </c>
       <c r="C151" t="s">
-        <v>462</v>
+        <v>471</v>
       </c>
       <c r="D151" t="s">
-        <v>105</v>
+        <v>472</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>463</v>
+        <v>473</v>
       </c>
       <c r="B152" t="s">
-        <v>413</v>
+        <v>455</v>
       </c>
       <c r="C152" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
       <c r="D152" t="s">
-        <v>465</v>
+        <v>105</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="B153" t="s">
-        <v>413</v>
+        <v>455</v>
       </c>
       <c r="C153" t="s">
-        <v>467</v>
+        <v>476</v>
       </c>
       <c r="D153" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B154" t="s">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="C154" t="s">
-        <v>470</v>
+        <v>480</v>
       </c>
       <c r="D154" t="s">
-        <v>471</v>
+        <v>481</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>472</v>
+        <v>482</v>
       </c>
       <c r="B155" t="s">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="C155" t="s">
-        <v>473</v>
+        <v>483</v>
       </c>
       <c r="D155" t="s">
-        <v>340</v>
+        <v>484</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="B156" t="s">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="C156" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
       <c r="D156" t="s">
-        <v>441</v>
+        <v>487</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>476</v>
+        <v>488</v>
       </c>
       <c r="B157" t="s">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="C157" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="D157" t="s">
-        <v>478</v>
+        <v>490</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
+        <v>491</v>
+      </c>
+      <c r="B158" t="s">
         <v>479</v>
       </c>
-      <c r="B158" t="s">
-        <v>413</v>
-      </c>
       <c r="C158" t="s">
-        <v>480</v>
+        <v>492</v>
       </c>
       <c r="D158" t="s">
-        <v>481</v>
+        <v>33</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="B159" t="s">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="C159" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
       <c r="D159" t="s">
-        <v>316</v>
+        <v>495</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>484</v>
+        <v>496</v>
       </c>
       <c r="B160" t="s">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="C160" t="s">
-        <v>485</v>
+        <v>497</v>
       </c>
       <c r="D160" t="s">
-        <v>486</v>
+        <v>498</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>487</v>
+        <v>499</v>
       </c>
       <c r="B161" t="s">
-        <v>413</v>
+        <v>479</v>
       </c>
       <c r="C161" t="s">
-        <v>488</v>
+        <v>500</v>
       </c>
       <c r="D161" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="B162" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C162" t="s">
-        <v>492</v>
+        <v>502</v>
       </c>
       <c r="D162" t="s">
-        <v>234</v>
+        <v>498</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>493</v>
+        <v>503</v>
       </c>
       <c r="B163" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C163" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
       <c r="D163" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="B164" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C164" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="D164" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="B165" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C165" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="D165" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="B166" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C166" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="D166" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="B167" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C167" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="D167" t="s">
-        <v>506</v>
+        <v>516</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>507</v>
+        <v>517</v>
       </c>
       <c r="B168" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C168" t="s">
-        <v>508</v>
+        <v>518</v>
       </c>
       <c r="D168" t="s">
-        <v>509</v>
+        <v>105</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>510</v>
+        <v>519</v>
       </c>
       <c r="B169" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C169" t="s">
-        <v>511</v>
+        <v>520</v>
       </c>
       <c r="D169" t="s">
-        <v>512</v>
+        <v>105</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="B170" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C170" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="D170" t="s">
-        <v>515</v>
+        <v>498</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="B171" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C171" t="s">
-        <v>517</v>
+        <v>524</v>
       </c>
       <c r="D171" t="s">
-        <v>518</v>
+        <v>105</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="B172" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C172" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="D172" t="s">
         <v>105</v>
@@ -4692,13 +5043,13 @@
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="B173" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C173" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="D173" t="s">
         <v>105</v>
@@ -4706,262 +5057,850 @@
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="B174" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C174" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D174" t="s">
-        <v>105</v>
+        <v>531</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
       <c r="B175" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C175" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="D175" t="s">
-        <v>105</v>
+        <v>534</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>527</v>
+        <v>535</v>
       </c>
       <c r="B176" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C176" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="D176" t="s">
-        <v>105</v>
+        <v>537</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>529</v>
+        <v>538</v>
       </c>
       <c r="B177" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="C177" t="s">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="D177" t="s">
-        <v>105</v>
+        <v>370</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>531</v>
+        <v>540</v>
       </c>
       <c r="B178" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C178" t="s">
-        <v>533</v>
+        <v>541</v>
       </c>
       <c r="D178" t="s">
-        <v>534</v>
+        <v>507</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="B179" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C179" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
       <c r="D179" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
       <c r="B180" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C180" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
       <c r="D180" t="s">
-        <v>537</v>
+        <v>547</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="B181" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C181" t="s">
-        <v>541</v>
+        <v>549</v>
       </c>
       <c r="D181" t="s">
-        <v>537</v>
+        <v>346</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="B182" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C182" t="s">
-        <v>543</v>
+        <v>551</v>
       </c>
       <c r="D182" t="s">
-        <v>544</v>
+        <v>552</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>545</v>
+        <v>553</v>
       </c>
       <c r="B183" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C183" t="s">
-        <v>546</v>
+        <v>554</v>
       </c>
       <c r="D183" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>547</v>
+        <v>556</v>
       </c>
       <c r="B184" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C184" t="s">
-        <v>548</v>
+        <v>557</v>
       </c>
       <c r="D184" t="s">
-        <v>544</v>
+        <v>558</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>549</v>
+        <v>559</v>
       </c>
       <c r="B185" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C185" t="s">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="D185" t="s">
-        <v>537</v>
+        <v>561</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="B186" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C186" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
       <c r="D186" t="s">
-        <v>544</v>
+        <v>564</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>553</v>
+        <v>565</v>
       </c>
       <c r="B187" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C187" t="s">
-        <v>554</v>
+        <v>566</v>
       </c>
       <c r="D187" t="s">
-        <v>544</v>
+        <v>105</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>555</v>
+        <v>567</v>
       </c>
       <c r="B188" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C188" t="s">
-        <v>556</v>
+        <v>568</v>
       </c>
       <c r="D188" t="s">
-        <v>537</v>
+        <v>105</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>557</v>
+        <v>569</v>
       </c>
       <c r="B189" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C189" t="s">
-        <v>558</v>
+        <v>570</v>
       </c>
       <c r="D189" t="s">
-        <v>537</v>
+        <v>547</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>559</v>
+        <v>571</v>
       </c>
       <c r="B190" t="s">
-        <v>532</v>
+        <v>479</v>
       </c>
       <c r="C190" t="s">
-        <v>560</v>
+        <v>572</v>
       </c>
       <c r="D190" t="s">
-        <v>537</v>
+        <v>246</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>561</v>
+        <v>573</v>
       </c>
       <c r="B191" t="s">
-        <v>532</v>
+        <v>574</v>
       </c>
       <c r="C191" t="s">
-        <v>562</v>
+        <v>575</v>
       </c>
       <c r="D191" t="s">
-        <v>537</v>
+        <v>234</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>576</v>
+      </c>
+      <c r="B192" t="s">
+        <v>574</v>
+      </c>
+      <c r="C192" t="s">
+        <v>577</v>
+      </c>
+      <c r="D192" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>579</v>
+      </c>
+      <c r="B193" t="s">
+        <v>574</v>
+      </c>
+      <c r="C193" t="s">
+        <v>580</v>
+      </c>
+      <c r="D193" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>582</v>
+      </c>
+      <c r="B194" t="s">
+        <v>574</v>
+      </c>
+      <c r="C194" t="s">
+        <v>583</v>
+      </c>
+      <c r="D194" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>585</v>
+      </c>
+      <c r="B195" t="s">
+        <v>574</v>
+      </c>
+      <c r="C195" t="s">
+        <v>586</v>
+      </c>
+      <c r="D195" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>588</v>
+      </c>
+      <c r="B196" t="s">
+        <v>574</v>
+      </c>
+      <c r="C196" t="s">
+        <v>589</v>
+      </c>
+      <c r="D196" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>590</v>
+      </c>
+      <c r="B197" t="s">
+        <v>574</v>
+      </c>
+      <c r="C197" t="s">
+        <v>591</v>
+      </c>
+      <c r="D197" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>593</v>
+      </c>
+      <c r="B198" t="s">
+        <v>574</v>
+      </c>
+      <c r="C198" t="s">
+        <v>594</v>
+      </c>
+      <c r="D198" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>596</v>
+      </c>
+      <c r="B199" t="s">
+        <v>574</v>
+      </c>
+      <c r="C199" t="s">
+        <v>597</v>
+      </c>
+      <c r="D199" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>599</v>
+      </c>
+      <c r="B200" t="s">
+        <v>574</v>
+      </c>
+      <c r="C200" t="s">
+        <v>600</v>
+      </c>
+      <c r="D200" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>602</v>
+      </c>
+      <c r="B201" t="s">
+        <v>574</v>
+      </c>
+      <c r="C201" t="s">
+        <v>603</v>
+      </c>
+      <c r="D201" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>604</v>
+      </c>
+      <c r="B202" t="s">
+        <v>574</v>
+      </c>
+      <c r="C202" t="s">
+        <v>605</v>
+      </c>
+      <c r="D202" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>606</v>
+      </c>
+      <c r="B203" t="s">
+        <v>574</v>
+      </c>
+      <c r="C203" t="s">
+        <v>607</v>
+      </c>
+      <c r="D203" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>608</v>
+      </c>
+      <c r="B204" t="s">
+        <v>574</v>
+      </c>
+      <c r="C204" t="s">
+        <v>609</v>
+      </c>
+      <c r="D204" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>610</v>
+      </c>
+      <c r="B205" t="s">
+        <v>574</v>
+      </c>
+      <c r="C205" t="s">
+        <v>611</v>
+      </c>
+      <c r="D205" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>612</v>
+      </c>
+      <c r="B206" t="s">
+        <v>574</v>
+      </c>
+      <c r="C206" t="s">
+        <v>613</v>
+      </c>
+      <c r="D206" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>614</v>
+      </c>
+      <c r="B207" t="s">
+        <v>615</v>
+      </c>
+      <c r="C207" t="s">
+        <v>616</v>
+      </c>
+      <c r="D207" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>618</v>
+      </c>
+      <c r="B208" t="s">
+        <v>615</v>
+      </c>
+      <c r="C208" t="s">
+        <v>619</v>
+      </c>
+      <c r="D208" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>621</v>
+      </c>
+      <c r="B209" t="s">
+        <v>615</v>
+      </c>
+      <c r="C209" t="s">
+        <v>622</v>
+      </c>
+      <c r="D209" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>623</v>
+      </c>
+      <c r="B210" t="s">
+        <v>615</v>
+      </c>
+      <c r="C210" t="s">
+        <v>624</v>
+      </c>
+      <c r="D210" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>625</v>
+      </c>
+      <c r="B211" t="s">
+        <v>615</v>
+      </c>
+      <c r="C211" t="s">
+        <v>626</v>
+      </c>
+      <c r="D211" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>628</v>
+      </c>
+      <c r="B212" t="s">
+        <v>615</v>
+      </c>
+      <c r="C212" t="s">
+        <v>629</v>
+      </c>
+      <c r="D212" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>630</v>
+      </c>
+      <c r="B213" t="s">
+        <v>615</v>
+      </c>
+      <c r="C213" t="s">
+        <v>631</v>
+      </c>
+      <c r="D213" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>632</v>
+      </c>
+      <c r="B214" t="s">
+        <v>615</v>
+      </c>
+      <c r="C214" t="s">
+        <v>633</v>
+      </c>
+      <c r="D214" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>634</v>
+      </c>
+      <c r="B215" t="s">
+        <v>615</v>
+      </c>
+      <c r="C215" t="s">
+        <v>635</v>
+      </c>
+      <c r="D215" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>636</v>
+      </c>
+      <c r="B216" t="s">
+        <v>615</v>
+      </c>
+      <c r="C216" t="s">
+        <v>637</v>
+      </c>
+      <c r="D216" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>638</v>
+      </c>
+      <c r="B217" t="s">
+        <v>615</v>
+      </c>
+      <c r="C217" t="s">
+        <v>639</v>
+      </c>
+      <c r="D217" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>640</v>
+      </c>
+      <c r="B218" t="s">
+        <v>615</v>
+      </c>
+      <c r="C218" t="s">
+        <v>641</v>
+      </c>
+      <c r="D218" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>642</v>
+      </c>
+      <c r="B219" t="s">
+        <v>615</v>
+      </c>
+      <c r="C219" t="s">
+        <v>643</v>
+      </c>
+      <c r="D219" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>644</v>
+      </c>
+      <c r="B220" t="s">
+        <v>615</v>
+      </c>
+      <c r="C220" t="s">
+        <v>645</v>
+      </c>
+      <c r="D220" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>646</v>
+      </c>
+      <c r="B221" t="s">
+        <v>647</v>
+      </c>
+      <c r="C221" t="s">
+        <v>648</v>
+      </c>
+      <c r="D221" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>650</v>
+      </c>
+      <c r="B222" t="s">
+        <v>647</v>
+      </c>
+      <c r="C222" t="s">
+        <v>651</v>
+      </c>
+      <c r="D222" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>652</v>
+      </c>
+      <c r="B223" t="s">
+        <v>647</v>
+      </c>
+      <c r="C223" t="s">
+        <v>653</v>
+      </c>
+      <c r="D223" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>655</v>
+      </c>
+      <c r="B224" t="s">
+        <v>647</v>
+      </c>
+      <c r="C224" t="s">
+        <v>656</v>
+      </c>
+      <c r="D224" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>658</v>
+      </c>
+      <c r="B225" t="s">
+        <v>647</v>
+      </c>
+      <c r="C225" t="s">
+        <v>659</v>
+      </c>
+      <c r="D225" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>661</v>
+      </c>
+      <c r="B226" t="s">
+        <v>647</v>
+      </c>
+      <c r="C226" t="s">
+        <v>662</v>
+      </c>
+      <c r="D226" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>664</v>
+      </c>
+      <c r="B227" t="s">
+        <v>647</v>
+      </c>
+      <c r="C227" t="s">
+        <v>665</v>
+      </c>
+      <c r="D227" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>666</v>
+      </c>
+      <c r="B228" t="s">
+        <v>647</v>
+      </c>
+      <c r="C228" t="s">
+        <v>667</v>
+      </c>
+      <c r="D228" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>669</v>
+      </c>
+      <c r="B229" t="s">
+        <v>647</v>
+      </c>
+      <c r="C229" t="s">
+        <v>670</v>
+      </c>
+      <c r="D229" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>671</v>
+      </c>
+      <c r="B230" t="s">
+        <v>647</v>
+      </c>
+      <c r="C230" t="s">
+        <v>672</v>
+      </c>
+      <c r="D230" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>673</v>
+      </c>
+      <c r="B231" t="s">
+        <v>674</v>
+      </c>
+      <c r="C231" t="s">
+        <v>675</v>
+      </c>
+      <c r="D231" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>676</v>
+      </c>
+      <c r="B232" t="s">
+        <v>674</v>
+      </c>
+      <c r="C232" t="s">
+        <v>677</v>
+      </c>
+      <c r="D232" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>678</v>
+      </c>
+      <c r="B233" t="s">
+        <v>674</v>
+      </c>
+      <c r="C233" t="s">
+        <v>679</v>
+      </c>
+      <c r="D233" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of: Pass, Fail, Blocked, N/A" sqref="E10:E191">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of: Pass, Fail, Blocked, N/A" sqref="E10:E233">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of: Pass, Fail, Blocked, N/A" sqref="E2:E191">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose one of: Pass, Fail, Blocked, N/A" sqref="E2:E233">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4984,55 +5923,55 @@
         <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>563</v>
+        <v>680</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>564</v>
+        <v>681</v>
       </c>
       <c r="B2">
-        <f>COUNTIF('Test Cases'!E2:E191,"Pass")</f>
+        <f>COUNTIF('Test Cases'!E2:E233,"Pass")</f>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>565</v>
+        <v>682</v>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Cases'!E2:E191,"Fail")</f>
+        <f>COUNTIF('Test Cases'!E2:E233,"Fail")</f>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>566</v>
+        <v>683</v>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Cases'!E2:E191,"Blocked")</f>
+        <f>COUNTIF('Test Cases'!E2:E233,"Blocked")</f>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>567</v>
+        <v>684</v>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Cases'!E2:E191,"N/A")</f>
+        <f>COUNTIF('Test Cases'!E2:E233,"N/A")</f>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>568</v>
+        <v>685</v>
       </c>
       <c r="B6">
-        <v>190</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>569</v>
+        <v>686</v>
       </c>
       <c r="B7">
-        <f>COUNTA('Test Cases'!E2:E191)</f>
+        <f>COUNTA('Test Cases'!E2:E233)</f>
       </c>
     </row>
   </sheetData>
@@ -5052,15 +5991,15 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>570</v>
+        <v>687</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>571</v>
+        <v>688</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>572</v>
+        <v>689</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -5068,7 +6007,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>573</v>
+        <v>690</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -5076,7 +6015,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>574</v>
+        <v>691</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
@@ -5084,7 +6023,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>575</v>
+        <v>692</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
@@ -5092,7 +6031,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>576</v>
+        <v>693</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
@@ -5100,7 +6039,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>577</v>
+        <v>694</v>
       </c>
       <c r="B8" t="s">
         <v>5</v>
@@ -5108,7 +6047,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>578</v>
+        <v>695</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
@@ -5116,7 +6055,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>579</v>
+        <v>696</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
@@ -5138,7 +6077,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>580</v>
+        <v>697</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -5148,27 +6087,27 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>581</v>
+        <v>698</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>582</v>
+        <v>699</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>583</v>
+        <v>700</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>584</v>
+        <v>701</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>585</v>
+        <v>702</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
@@ -5178,7 +6117,7 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>586</v>
+        <v>703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>